<commit_message>
adiciona logica buscar email cielo e bradesco
</commit_message>
<xml_diff>
--- a/ID01_1_ConcEst_Download/resources/config/Config.xlsx
+++ b/ID01_1_ConcEst_Download/resources/config/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RPA\ID01_1_ConcEst_Download\ID01_1_ConcEst_Download\resources\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C84C2DCE-EBAA-4174-A6C3-2B4B9FC3F2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6AAAC84-5722-4724-BBB1-A49F269C9AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="120">
   <si>
     <t>Name</t>
   </si>
@@ -380,13 +380,16 @@
   </si>
   <si>
     <t>arquivos_baixados</t>
+  </si>
+  <si>
+    <t>mmorais@aifastlab.site</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -426,6 +429,14 @@
       <color theme="1"/>
       <name val="Aptos"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -473,10 +484,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -515,8 +527,12 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -986,7 +1002,9 @@
       <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="7"/>
+      <c r="B9" s="7" t="s">
+        <v>115</v>
+      </c>
       <c r="C9" s="5" t="s">
         <v>25</v>
       </c>
@@ -995,7 +1013,9 @@
       <c r="A10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="8"/>
+      <c r="B10" s="14" t="s">
+        <v>119</v>
+      </c>
       <c r="C10" s="5" t="s">
         <v>27</v>
       </c>
@@ -4221,8 +4241,11 @@
       <c r="B990" s="4"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B10" r:id="rId1" xr:uid="{CE890819-87C4-4EDF-BB6A-F4520053B963}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>